<commit_message>
adjust tabla carga masiva
</commit_message>
<xml_diff>
--- a/Backend/TablaCargaMasiva.xlsx
+++ b/Backend/TablaCargaMasiva.xlsx
@@ -49,7 +49,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
       </patternFill>
     </fill>
     <fill>
@@ -98,21 +103,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -478,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -495,6 +503,10 @@
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -568,342 +580,498 @@
           <t>related_product_codes</t>
         </is>
       </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>is_specs_column</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>spec_1</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>spec_2</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>spec_3</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>MAT-001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Matraz Aforado Clase A</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>LabEquip</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>equipos</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Material Volumetrico</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Matraces</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Matraz aforado de vidrio borosilicato clase A</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>matraz_aforado.jpg</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>velocidad</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>MAT-001</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>MAT-001-25ML</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>25 ml</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>70x40mm</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="N3" s="4" t="n"/>
+      <c r="O3" s="4" t="n"/>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>20hp</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>25mhp</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>25ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>MAT-001</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>MAT-001-50ML</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>90x45mm</t>
         </is>
       </c>
-      <c r="N3" s="3" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="N4" s="4" t="n"/>
+      <c r="O4" s="4" t="n"/>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>40hp</t>
+        </is>
+      </c>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>30mhp</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>50ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>MAT-001</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>MAT-001-100ML</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>110x50mm</t>
         </is>
       </c>
-      <c r="N4" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>60hp</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>40mhp</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>100ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
+      <c r="N6" s="3" t="n"/>
+      <c r="O6" s="3" t="n"/>
+      <c r="P6" s="3" t="n"/>
+      <c r="Q6" s="3" t="n"/>
+      <c r="R6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>VAS-002</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Vaso de Precipitado</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>GlassLab</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>equipos</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Cristaleria</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Vaso de precipitado graduado</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>vaso_precipitado.jpg</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>MAT-001</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>MAT-001-250ML</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>viscosidad</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>dimensiones</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>VAS-002</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>VAS-002-100ML</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>100 ml</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>50x70mm</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="n"/>
+      <c r="O8" s="4" t="n"/>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>52cP</t>
+        </is>
+      </c>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>50x70mm</t>
+        </is>
+      </c>
+      <c r="R8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>VAS-002</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>VAS-002-250ML</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>250 ml</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>140x60mm</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>70x95mm</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="n"/>
+      <c r="O9" s="4" t="n"/>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>48cP</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>70x95mm</t>
+        </is>
+      </c>
+      <c r="R9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>VAS-002</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Vaso de Precipitado</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>GlassLab</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>equipos</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Cristaleria</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Vasos</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Vaso de precipitado graduado</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>vaso_precipitado.jpg</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>VAS-002-100ML</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>100 ml</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>50x70mm</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>MAT-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>VAS-002</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>VAS-002-250ML</t>
-        </is>
-      </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>250 ml</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>70x95mm</t>
-        </is>
-      </c>
-      <c r="N8" s="3" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>VAS-002</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>VAS-002-500ML</t>
         </is>
       </c>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>500 ml</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>90x125mm</t>
         </is>
       </c>
-      <c r="N9" s="3" t="n"/>
+      <c r="N10" s="4" t="n"/>
+      <c r="O10" s="4" t="n"/>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>45cP</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>90x125mm</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -916,357 +1084,448 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>INSTRUCCIONES PARA CARGA MASIVA CON VARIANTES</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr"/>
+      <c r="A2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>1. COLUMNAS DISPONIBLES</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   product_code          Codigo unico del producto (obligatorio)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   name                  Nombre del producto</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   brand                 Marca del producto</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   category_level_0      Categoria raiz: insumos, procesos, equipos, mobiliario (obligatoria si hay categoria)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   category_level_1      Subcategoria nivel 1 (se crea si no existe)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   category_level_2      Subcategoria nivel 2 (se crea si no existe, requiere level_1)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   description           Descripcion del producto</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   image_name            Nombre del archivo de imagen en la libreria (ej: producto.jpg)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   is_active             true/false - si el producto esta activo (default: true)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   is_variant            true/false - si la fila es una variante o un producto</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   variant_code          Codigo unico de la variante (obligatorio para variantes)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   variant_name          Nombre de la variante (ej: 250 ml, Talla L, Version A)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   dimensions            Dimensiones fisicas (ej: 10x5x5cm, 70x40mm)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   related_product_codes Codigos de productos relacionados separados por ; (ej: MAT-001;VAS-002)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   is_specs_column       true/false - si las variantes del producto tendran TechnicalSpecs dinamicas</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>2. CREAR UN PRODUCTO CON VARIANTES</t>
+          <t xml:space="preserve">   [columnas dinamicas]  Cualquier columna despues de is_specs_column es un TechnicalSpec.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Paso 1: En la primera fila del producto, completar name, brand, category, etc. con is_variant=false</t>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                         El nombre de la columna = key, el valor de la celda = value.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Paso 2: Para cada variante del mismo producto, usar el mismo product_code con is_variant=true</t>
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                         Ejemplo: agregar columna "potencia" con valor "20hp" en la variante.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Paso 3: Completar variant_code y variant_name en cada fila (de producto y de variante)</t>
-        </is>
-      </c>
+      <c r="A22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>2. TECHNICAL SPECS DINAMICAS</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   NOTA: Las especificaciones tecnicas dinamicas (voltaje, material, presion, etc.)</t>
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Solo aplican a variantes (is_variant=true), nunca al producto padre</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   se gestionan desde el panel de administracion o via API (/products/technical-specs/)</t>
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - El producto padre define is_specs_column=true para habilitar el procesamiento</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   y no forman parte de la carga masiva CSV/Excel.</t>
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Agregar tantas columnas dinamicas como necesites despues de is_specs_column</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr"/>
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Si el valor esta vacio, igual se crea el TechnicalSpec con value=""</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>3. REGLAS</t>
+          <t xml:space="preserve">   - Al reimportar una variante existente, sus specs anteriores se reemplazan por las nuevas</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Solo puede haber UN producto (is_variant=false) por product_code</t>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Los nombres de columna dinamicas son libres (ej: potencia, velocidad, material, voltaje)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Las variantes (is_variant=true) DEBEN tener un producto padre existente o creado en el mismo archivo</t>
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Las columnas dinamicas en el Excel aplican a TODOS los productos del archivo.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Las variantes pueden dejar vacios los campos del producto (name, brand, category, etc.)</t>
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Si un producto no usa specs (is_specs_column=false), esas columnas se ignoran para el.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Cada variante debe tener un variant_code unico dentro del mismo producto</t>
-        </is>
-      </c>
+      <c r="A32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Si variant_code esta vacio, la fila no crea variante (se ignora esa parte)</t>
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>3. CREAR UN PRODUCTO CON VARIANTES</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr"/>
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Paso 1: Fila del producto (is_variant=false): completar name, brand, category, is_specs_column</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>4. EJEMPLO</t>
+          <t xml:space="preserve">   Paso 2: Para cada variante, usar el mismo product_code con is_variant=true</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   product_code | name       | ... | is_variant | variant_code  | variant_name | dimensions</t>
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Paso 3: Completar variant_code, variant_name y las columnas dinamicas en cada variante</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   MAT-001      | Matraz ... | ... | false      | MAT-001-25ML  | 25 ml        | 70x40mm</t>
-        </is>
-      </c>
+      <c r="A37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   MAT-001      |            | ... | true       | MAT-001-50ML  | 50 ml        | 90x45mm</t>
+          <t>4. REGLAS</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   MAT-001      |            | ... | true       | MAT-001-100ML | 100 ml       | 110x50mm</t>
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Solo puede haber UN producto (is_variant=false) por product_code</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr"/>
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Las variantes (is_variant=true) DEBEN tener un producto padre existente o creado en el mismo archivo</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>5. ERRORES COMUNES</t>
+          <t xml:space="preserve">   - Las variantes pueden dejar vacios los campos del producto (name, brand, category, etc.)</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Cada variante debe tener un variant_code unico dentro del mismo producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Si variant_code esta vacio, la fila no crea variante (se ignora esa parte)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>5. EJEMPLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   product_code | ... | is_variant | variant_code  | is_specs_column | spec_1     | spec_2    | spec_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MAT-001      | ... | false      |               | true            | potencia   | velocidad | volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MAT-001      | ... | true       | MAT-001-25ML  |                 | 20hp       | 25mhp     | 25ml  </t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MAT-001      | ... | true       | MAT-001-50ML  |                 | 40hp       | 30mhp     | 50ml  </t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   VAS-002      | ... | false      |               | true            | viscosidad | dimensiones |     </t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   VAS-002      | ... | true       | VAS-002-100ML |                 | 52cP       | 50x70mm     |     </t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>6. ERRORES COMUNES</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - Variante (is_variant=true) sin product_code: fila ignorada con error</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - Variante (is_variant=true) sin variant_code: fila ignorada con error</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - Mas de un producto con el mismo product_code (is_variant=false): segundo es ignorado con error</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - Variante cuyo product_code no existe en DB ni en el archivo: error</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>6. CAMBIOS RESPECTO A LA VERSION ANTERIOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>7. CAMBIOS RESPECTO A LA VERSION ANTERIOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - spec_code         =&gt; variant_code  (renombrado)</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - volume            =&gt; variant_name  (renombrado, ahora es el nombre descriptivo de la variante)</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - cap               =&gt; ELIMINADO (manejar via TechnicalSpecs en admin/API)</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - outlet            =&gt; ELIMINADO (manejar via TechnicalSpecs en admin/API)</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - accuracy          =&gt; ELIMINADO (manejar via TechnicalSpecs en admin/API)</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - precision         =&gt; ELIMINADO (manejar via TechnicalSpecs en admin/API)</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   - additional_specs  =&gt; ELIMINADO (manejar via TechnicalSpecs en admin/API)</t>
         </is>

</xml_diff>

<commit_message>
implementacion de  mejoras carga  masiva
</commit_message>
<xml_diff>
--- a/Backend/TablaCargaMasiva.xlsx
+++ b/Backend/TablaCargaMasiva.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +48,13 @@
       <color rgb="008B0000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +79,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -121,6 +131,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,21 +500,21 @@
   <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
@@ -512,77 +523,77 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>product_code</t>
+          <t>codigo_producto</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>nombre</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>brand</t>
+          <t>marca</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>category_level_0</t>
+          <t>categoria_nivel_0</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>category_level_1</t>
+          <t>categoria_nivel_1</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>category_level_2</t>
+          <t>categoria_nivel_2</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>descripcion</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>image_name</t>
+          <t>nombre_imagen</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>activo</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>is_variant</t>
+          <t>es_variante</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>variant_code</t>
+          <t>codigo_variante</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>variant_name</t>
+          <t>nombre_variante</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>dimensions</t>
+          <t>dimensiones</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>related_product_codes</t>
+          <t>productos_relacionados</t>
         </is>
       </c>
       <c r="O1" s="2" t="inlineStr">
         <is>
-          <t>is_specs_column</t>
+          <t>tiene_specs</t>
         </is>
       </c>
       <c r="P1" s="2" t="inlineStr">
@@ -924,7 +935,7 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>dimensiones</t>
+          <t>cap_nominal</t>
         </is>
       </c>
       <c r="R7" s="3" t="n"/>
@@ -972,7 +983,7 @@
       </c>
       <c r="Q8" s="4" t="inlineStr">
         <is>
-          <t>50x70mm</t>
+          <t>100ml</t>
         </is>
       </c>
       <c r="R8" s="4" t="n"/>
@@ -1020,7 +1031,7 @@
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
-          <t>70x95mm</t>
+          <t>250ml</t>
         </is>
       </c>
       <c r="R9" s="4" t="n"/>
@@ -1068,7 +1079,7 @@
       </c>
       <c r="Q10" s="4" t="inlineStr">
         <is>
-          <t>90x125mm</t>
+          <t>500ml</t>
         </is>
       </c>
       <c r="R10" s="4" t="n"/>
@@ -1084,16 +1095,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A67"/>
+  <dimension ref="A1:A88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="115" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>INSTRUCCIONES PARA CARGA MASIVA CON VARIANTES</t>
+          <t>INSTRUCCIONES PARA CARGA MASIVA DE PRODUCTOS Y VARIANTES</t>
         </is>
       </c>
     </row>
@@ -1110,424 +1121,543 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   product_code          Codigo unico del producto (obligatorio)</t>
+          <t xml:space="preserve">   codigo_producto        Codigo unico del producto (obligatorio)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   name                  Nombre del producto</t>
+          <t xml:space="preserve">   nombre                 Nombre del producto</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   brand                 Marca del producto</t>
+          <t xml:space="preserve">   marca                  Marca del producto</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   category_level_0      Categoria raiz: insumos, procesos, equipos, mobiliario (obligatoria si hay categoria)</t>
+          <t xml:space="preserve">   categoria_nivel_0      Categoria raiz — valores validos: insumos, procesos, equipos, mobiliario</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   category_level_1      Subcategoria nivel 1 (se crea si no existe)</t>
+          <t xml:space="preserve">   categoria_nivel_1      Subcategoria nivel 1 (se crea si no existe)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   category_level_2      Subcategoria nivel 2 (se crea si no existe, requiere level_1)</t>
+          <t xml:space="preserve">   categoria_nivel_2      Subcategoria nivel 2 (se crea si no existe; requiere categoria_nivel_1)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   description           Descripcion del producto</t>
+          <t xml:space="preserve">   descripcion            Descripcion del producto</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   image_name            Nombre del archivo de imagen en la libreria (ej: producto.jpg)</t>
+          <t xml:space="preserve">   nombre_imagen          Nombre del archivo de imagen en la libreria (ej: producto.jpg)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   is_active             true/false - si el producto esta activo (default: true)</t>
+          <t xml:space="preserve">   activo                 true/false — si el producto esta activo (por defecto: true)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   is_variant            true/false - si la fila es una variante o un producto</t>
+          <t xml:space="preserve">   es_variante            true/false — si la fila es una variante (true) o un producto padre (false)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   variant_code          Codigo unico de la variante (obligatorio para variantes)</t>
+          <t xml:space="preserve">   codigo_variante        Codigo unico de la variante (obligatorio para es_variante=true)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   variant_name          Nombre de la variante (ej: 250 ml, Talla L, Version A)</t>
+          <t xml:space="preserve">   nombre_variante        Nombre descriptivo de la variante (ej: 250 ml, Talla L)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   dimensions            Dimensiones fisicas (ej: 10x5x5cm, 70x40mm)</t>
+          <t xml:space="preserve">   dimensiones            Dimensiones fisicas (ej: 10x5x5cm, 70x40mm)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   related_product_codes Codigos de productos relacionados separados por ; (ej: MAT-001;VAS-002)</t>
+          <t xml:space="preserve">   productos_relacionados Codigos de productos relacionados separados por ; (ej: MAT-001;VAS-002)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   is_specs_column       true/false - si las variantes del producto tendran TechnicalSpecs dinamicas</t>
+          <t xml:space="preserve">   tiene_specs            true/false — en la fila del producto padre: habilita specs dinamicas para sus variantes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   [columnas dinamicas]  Cualquier columna despues de is_specs_column es un TechnicalSpec.</t>
+          <t xml:space="preserve">   spec_1, spec_2, ...    Columnas de specs dinamicas: el padre escribe el NOMBRE, la variante escribe el VALOR</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                         El nombre de la columna = key, el valor de la celda = value.</t>
-        </is>
-      </c>
+      <c r="A20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                         Ejemplo: agregar columna "potencia" con valor "20hp" en la variante.</t>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>2. SPECS DINAMICAS DE VARIANTES</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr"/>
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Solo aplican a variantes (es_variante=true), nunca al producto padre</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>2. TECHNICAL SPECS DINAMICAS</t>
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - En la fila del producto padre, escribir el NOMBRE de cada atributo (ej: potencia, material)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Solo aplican a variantes (is_variant=true), nunca al producto padre</t>
+          <t xml:space="preserve">   - En cada fila de variante, escribir el VALOR correspondiente (ej: 20hp, acero inoxidable)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - El producto padre define is_specs_column=true para habilitar el procesamiento</t>
+          <t xml:space="preserve">   - Columnas sin nombre en la fila del padre se ignoran completamente</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Agregar tantas columnas dinamicas como necesites despues de is_specs_column</t>
+          <t xml:space="preserve">   - Al reimportar una variante existente, sus specs anteriores se reemplazan por las nuevas</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Si el valor esta vacio, igual se crea el TechnicalSpec con value=""</t>
+          <t xml:space="preserve">   - Podes agregar tantas columnas de specs como necesites (spec_1, spec_2, spec_3, ...)</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Al reimportar una variante existente, sus specs anteriores se reemplazan por las nuevas</t>
-        </is>
-      </c>
+      <c r="A28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Los nombres de columna dinamicas son libres (ej: potencia, velocidad, material, voltaje)</t>
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>3. PASOS PARA CARGAR UN PRODUCTO CON VARIANTES</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Las columnas dinamicas en el Excel aplican a TODOS los productos del archivo.</t>
+          <t xml:space="preserve">   Paso 1: Una fila con es_variante=false define el producto padre (nombre, marca, categoria, etc.)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Si un producto no usa specs (is_specs_column=false), esas columnas se ignoran para el.</t>
+          <t xml:space="preserve">          Si usa specs, poner tiene_specs=true y escribir los nombres de atributos en spec_1, spec_2...</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr"/>
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Paso 2: Para cada variante, una fila con es_variante=true y el mismo codigo_producto</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>3. CREAR UN PRODUCTO CON VARIANTES</t>
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Completar codigo_variante, nombre_variante y los valores de specs</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Paso 1: Fila del producto (is_variant=false): completar name, brand, category, is_specs_column</t>
-        </is>
-      </c>
+      <c r="A34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Paso 2: Para cada variante, usar el mismo product_code con is_variant=true</t>
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>4. EJEMPLO</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Paso 3: Completar variant_code, variant_name y las columnas dinamicas en cada variante</t>
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   codigo_producto | es_variante | codigo_variante | tiene_specs | spec_1   | spec_2   </t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr"/>
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MAT-001         | false       |                 | true        | potencia | volumen  </t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>4. REGLAS</t>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MAT-001         | true        | MAT-001-25ML    |             | 20hp     | 25ml     </t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Solo puede haber UN producto (is_variant=false) por product_code</t>
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MAT-001         | true        | MAT-001-50ML    |             | 40hp     | 50ml     </t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Las variantes (is_variant=true) DEBEN tener un producto padre existente o creado en el mismo archivo</t>
-        </is>
-      </c>
+      <c r="A40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Las variantes pueden dejar vacios los campos del producto (name, brand, category, etc.)</t>
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>5. ERRORES POSIBLES Y SOLUCIONES</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Cada variante debe tener un variant_code unico dentro del mismo producto</t>
-        </is>
-      </c>
+      <c r="A42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Si variant_code esta vacio, la fila no crea variante (se ignora esa parte)</t>
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ERROR: Fila N: variante sin codigo_producto</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="inlineStr"/>
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Causa:    La fila tiene es_variante=true pero no tiene codigo_producto.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>5. EJEMPLO</t>
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Solucion: Completar el campo codigo_producto con el codigo del producto padre.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   product_code | ... | is_variant | variant_code  | is_specs_column | spec_1     | spec_2    | spec_3</t>
-        </is>
-      </c>
+      <c r="A46" s="6" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   MAT-001      | ... | false      |               | true            | potencia   | velocidad | volumen</t>
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ERROR: Fila N: codigo_producto "X" duplicado</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   MAT-001      | ... | true       | MAT-001-25ML  |                 | 20hp       | 25mhp     | 25ml  </t>
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Causa:    Hay dos o mas filas con es_variante=false y el mismo codigo_producto.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   MAT-001      | ... | true       | MAT-001-50ML  |                 | 40hp       | 30mhp     | 50ml  </t>
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Solucion: Solo puede haber UNA fila de producto por codigo. Las demas deben ser variantes.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ---</t>
-        </is>
-      </c>
+      <c r="A50" s="6" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   VAS-002      | ... | false      |               | true            | viscosidad | dimensiones |     </t>
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ERROR: Fila N: variante sin codigo_variante</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   VAS-002      | ... | true       | VAS-002-100ML |                 | 52cP       | 50x70mm     |     </t>
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Causa:    La fila tiene es_variante=true pero no tiene codigo_variante.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr"/>
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Solucion: Completar el campo codigo_variante con un codigo unico para esa variante.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>6. ERRORES COMUNES</t>
-        </is>
-      </c>
+      <c r="A54" s="6" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Variante (is_variant=true) sin product_code: fila ignorada con error</t>
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ERROR: Fila N: producto padre con codigo_producto "X" no encontrado</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Variante (is_variant=true) sin variant_code: fila ignorada con error</t>
+          <t xml:space="preserve">   Causa:    La variante referencia un producto que no existe en la DB ni en el archivo.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Mas de un producto con el mismo product_code (is_variant=false): segundo es ignorado con error</t>
+          <t xml:space="preserve">   Solucion: Agregar la fila del producto padre en el mismo archivo, o verificar el codigo.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Variante cuyo product_code no existe en DB ni en el archivo: error</t>
-        </is>
-      </c>
+      <c r="A58" s="6" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr"/>
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ERROR: Fila N: imagen "X" no encontrada en la libreria de archivos</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>7. CAMBIOS RESPECTO A LA VERSION ANTERIOR</t>
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Causa:    El nombre_imagen no coincide con ningun archivo en la libreria de imagenes.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - spec_code         =&gt; variant_code  (renombrado)</t>
+          <t xml:space="preserve">   Solucion: Subir la imagen a la libreria antes de importar, o dejar el campo vacio.</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - volume            =&gt; variant_name  (renombrado, ahora es el nombre descriptivo de la variante)</t>
-        </is>
-      </c>
+      <c r="A62" s="6" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - cap               =&gt; ELIMINADO (manejar via TechnicalSpecs en admin/API)</t>
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ERROR: Fila N: error al procesar producto "X" — Categoria nivel 0 invalida</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - outlet            =&gt; ELIMINADO (manejar via TechnicalSpecs en admin/API)</t>
+          <t xml:space="preserve">   Causa:    El valor de categoria_nivel_0 no es uno de los permitidos.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - accuracy          =&gt; ELIMINADO (manejar via TechnicalSpecs en admin/API)</t>
+          <t xml:space="preserve">   Solucion: Usar solo: insumos, procesos, equipos, mobiliario (exactamente, sin tildes).</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - precision         =&gt; ELIMINADO (manejar via TechnicalSpecs en admin/API)</t>
-        </is>
-      </c>
+      <c r="A66" s="6" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - additional_specs  =&gt; ELIMINADO (manejar via TechnicalSpecs en admin/API)</t>
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ERROR: Fila N: producto relacionado con codigo "X" no encontrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Causa:    Un codigo en productos_relacionados no existe en la DB ni en el archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Solucion: Verificar el codigo o definir el producto relacionado en el mismo archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   NOTA: Si descargaste el Excel de errores y lo corregiste para reimportar,</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">         la columna "error" se ignora automaticamente — no hace falta borrarla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>6. CAMBIOS DE NOMBRES DE COLUMNAS (version anterior → actual)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   product_code         =&gt; codigo_producto</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   name                 =&gt; nombre</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   brand                =&gt; marca</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   category_level_0/1/2 =&gt; categoria_nivel_0/1/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   description          =&gt; descripcion</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   image_name           =&gt; nombre_imagen</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   is_active            =&gt; activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   is_variant           =&gt; es_variante</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   variant_code         =&gt; codigo_variante</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   variant_name         =&gt; nombre_variante</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   dimensions           =&gt; dimensiones</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   related_product_codes =&gt; productos_relacionados</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   is_specs_column      =&gt; tiene_specs</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (ambos formatos son aceptados por el importador)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add categ 3 en CM, delete dimensions, fix buscadores, fix orden technical spcec
</commit_message>
<xml_diff>
--- a/Backend/TablaCargaMasiva.xlsx
+++ b/Backend/TablaCargaMasiva.xlsx
@@ -506,13 +506,13 @@
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
@@ -553,37 +553,37 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>categoria_nivel_3</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>nombre_imagen</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>activo</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>es_variante</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>codigo_variante</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>nombre_variante</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>dimensiones</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
@@ -643,27 +643,27 @@
           <t>Matraces</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Matraz aforado de vidrio borosilicato clase A</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>matraz_aforado.jpg</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="K2" s="3" t="n"/>
       <c r="L2" s="3" t="n"/>
       <c r="M2" s="3" t="n"/>
       <c r="N2" s="3" t="n"/>
@@ -702,24 +702,20 @@
       <c r="G3" s="4" t="n"/>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="n"/>
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>MAT-001-25ML</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>25 ml</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>70x40mm</t>
         </is>
       </c>
       <c r="N3" s="4" t="n"/>
@@ -754,24 +750,20 @@
       <c r="G4" s="4" t="n"/>
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>MAT-001-50ML</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>50 ml</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>90x45mm</t>
         </is>
       </c>
       <c r="N4" s="4" t="n"/>
@@ -806,24 +798,20 @@
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>MAT-001-100ML</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>100 ml</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>110x50mm</t>
         </is>
       </c>
       <c r="N5" s="4" t="n"/>
@@ -895,27 +883,27 @@
           <t>Vasos</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Vaso de precipitado graduado</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>vaso_precipitado.jpg</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="K7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
       <c r="M7" s="3" t="n"/>
       <c r="N7" s="3" t="inlineStr">
@@ -954,24 +942,20 @@
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n"/>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>VAS-002-100ML</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>100 ml</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>50x70mm</t>
         </is>
       </c>
       <c r="N8" s="4" t="n"/>
@@ -1002,24 +986,20 @@
       <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="4" t="n"/>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="n"/>
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>VAS-002-250ML</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>250 ml</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>70x95mm</t>
         </is>
       </c>
       <c r="N9" s="4" t="n"/>
@@ -1050,24 +1030,20 @@
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="4" t="n"/>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>VAS-002-500ML</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>500 ml</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="inlineStr">
-        <is>
-          <t>90x125mm</t>
         </is>
       </c>
       <c r="N10" s="4" t="n"/>
@@ -1100,7 +1076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A88"/>
+  <dimension ref="A1:A87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -1168,49 +1144,49 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   descripcion            Descripcion del producto</t>
+          <t xml:space="preserve">   categoria_nivel_3      Subcategoria nivel 3 (se crea si no existe; requiere categoria_nivel_2)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   nombre_imagen          Nombre del archivo de imagen en la libreria (ej: producto.jpg)</t>
+          <t xml:space="preserve">   descripcion            Descripcion del producto</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   activo                 true/false — si el producto esta activo (por defecto: true)</t>
+          <t xml:space="preserve">   nombre_imagen          Nombre del archivo de imagen en la libreria (ej: producto.jpg)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   es_variante            true/false — si la fila es una variante (true) o un producto padre (false)</t>
+          <t xml:space="preserve">   activo                 true/false — si el producto esta activo (por defecto: true)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   codigo_variante        Codigo unico de la variante (obligatorio para es_variante=true)</t>
+          <t xml:space="preserve">   es_variante            true/false — si la fila es una variante (true) o un producto padre (false)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   nombre_variante        Nombre descriptivo de la variante (ej: 250 ml, Talla L)</t>
+          <t xml:space="preserve">   codigo_variante        Codigo unico de la variante (obligatorio para es_variante=true)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   dimensiones            Dimensiones fisicas (ej: 10x5x5cm, 70x40mm)</t>
+          <t xml:space="preserve">   nombre_variante        Nombre descriptivo de la variante (ej: 250 ml, Talla L)</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1568,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   category_level_0/1/2 =&gt; categoria_nivel_0/1/2</t>
+          <t xml:space="preserve">   category_level_0/1/2/3 =&gt; categoria_nivel_0/1/2/3</t>
         </is>
       </c>
     </row>
@@ -1641,26 +1617,19 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   dimensions           =&gt; dimensiones</t>
+          <t xml:space="preserve">   related_product_codes =&gt; productos_relacionados</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   related_product_codes =&gt; productos_relacionados</t>
+          <t xml:space="preserve">   is_specs_column      =&gt; tiene_specs</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   is_specs_column      =&gt; tiene_specs</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   (ambos formatos son aceptados por el importador)</t>
         </is>

</xml_diff>

<commit_message>
Revert "Revert "Consumibles back""
This reverts commit 24a3c0fdd1f65fc736f11074da92fd490d6e4b15.

ok
</commit_message>
<xml_diff>
--- a/Backend/TablaCargaMasiva.xlsx
+++ b/Backend/TablaCargaMasiva.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="233">
   <si>
     <t xml:space="preserve">codigo_producto</t>
   </si>
@@ -48,6 +48,21 @@
   </si>
   <si>
     <t xml:space="preserve">nombre_imagen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">articulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedronar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">archivo_esp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">archivo_hds</t>
   </si>
   <si>
     <t xml:space="preserve">activo</t>
@@ -995,8 +1010,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:DJ10"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:DO10"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
@@ -1004,12 +1019,15 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="114" min="15" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="119" min="20" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1052,19 +1070,19 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="2" t="s">
@@ -1355,58 +1373,73 @@
       <c r="DJ1" s="2" t="s">
         <v>113</v>
       </c>
+      <c r="DK1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="DL1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="DM1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="DN1" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="DO1" s="2" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>123</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
-      <c r="N2" s="3" t="s">
-        <v>122</v>
-      </c>
+      <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>126</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
+      <c r="S2" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
       <c r="Y2" s="3"/>
@@ -1499,10 +1532,15 @@
       <c r="DH2" s="3"/>
       <c r="DI2" s="3"/>
       <c r="DJ2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK2" s="3"/>
+      <c r="DL2" s="3"/>
+      <c r="DM2" s="3"/>
+      <c r="DN2" s="3"/>
+      <c r="DO2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -1513,28 +1551,28 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
-      <c r="K3" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>127</v>
-      </c>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
-      <c r="O3" s="4" t="s">
-        <v>128</v>
-      </c>
+      <c r="O3" s="4"/>
       <c r="P3" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
+      <c r="T3" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>135</v>
+      </c>
       <c r="W3" s="4"/>
       <c r="X3" s="4"/>
       <c r="Y3" s="4"/>
@@ -1627,10 +1665,15 @@
       <c r="DH3" s="4"/>
       <c r="DI3" s="4"/>
       <c r="DJ3" s="4"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK3" s="4"/>
+      <c r="DL3" s="4"/>
+      <c r="DM3" s="4"/>
+      <c r="DN3" s="4"/>
+      <c r="DO3" s="4"/>
+    </row>
+    <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -1641,28 +1684,28 @@
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
-      <c r="K4" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>131</v>
-      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
-      <c r="O4" s="4" t="s">
-        <v>132</v>
-      </c>
+      <c r="O4" s="4"/>
       <c r="P4" s="4" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
-      <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
-      <c r="V4" s="4"/>
+      <c r="T4" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="U4" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="V4" s="4" t="s">
+        <v>139</v>
+      </c>
       <c r="W4" s="4"/>
       <c r="X4" s="4"/>
       <c r="Y4" s="4"/>
@@ -1755,10 +1798,15 @@
       <c r="DH4" s="4"/>
       <c r="DI4" s="4"/>
       <c r="DJ4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK4" s="4"/>
+      <c r="DL4" s="4"/>
+      <c r="DM4" s="4"/>
+      <c r="DN4" s="4"/>
+      <c r="DO4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -1769,28 +1817,28 @@
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
-      <c r="K5" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>135</v>
-      </c>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
-      <c r="O5" s="4" t="s">
-        <v>136</v>
-      </c>
+      <c r="O5" s="4"/>
       <c r="P5" s="4" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
+      <c r="T5" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="V5" s="4" t="s">
+        <v>143</v>
+      </c>
       <c r="W5" s="4"/>
       <c r="X5" s="4"/>
       <c r="Y5" s="4"/>
@@ -1883,8 +1931,13 @@
       <c r="DH5" s="4"/>
       <c r="DI5" s="4"/>
       <c r="DJ5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK5" s="4"/>
+      <c r="DL5" s="4"/>
+      <c r="DM5" s="4"/>
+      <c r="DN5" s="4"/>
+      <c r="DO5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1999,57 +2052,62 @@
       <c r="DH6" s="3"/>
       <c r="DI6" s="3"/>
       <c r="DJ6" s="3"/>
+      <c r="DK6" s="3"/>
+      <c r="DL6" s="3"/>
+      <c r="DM6" s="3"/>
+      <c r="DN6" s="3"/>
+      <c r="DO6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>123</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
       <c r="L7" s="3"/>
-      <c r="M7" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>122</v>
-      </c>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
       <c r="O7" s="3" t="s">
-        <v>147</v>
+        <v>127</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>148</v>
+        <v>128</v>
       </c>
       <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
+      <c r="R7" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="S7" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="T7" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="U7" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
@@ -2143,10 +2201,15 @@
       <c r="DH7" s="3"/>
       <c r="DI7" s="3"/>
       <c r="DJ7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK7" s="3"/>
+      <c r="DL7" s="3"/>
+      <c r="DM7" s="3"/>
+      <c r="DN7" s="3"/>
+      <c r="DO7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -2157,25 +2220,25 @@
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
-      <c r="K8" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>149</v>
-      </c>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
-      <c r="O8" s="4" t="s">
-        <v>150</v>
-      </c>
+      <c r="O8" s="4"/>
       <c r="P8" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="Q8" s="4"/>
+        <v>127</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>154</v>
+      </c>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
-      <c r="T8" s="4"/>
-      <c r="U8" s="4"/>
+      <c r="T8" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="U8" s="4" t="s">
+        <v>143</v>
+      </c>
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
       <c r="X8" s="4"/>
@@ -2269,10 +2332,15 @@
       <c r="DH8" s="4"/>
       <c r="DI8" s="4"/>
       <c r="DJ8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK8" s="4"/>
+      <c r="DL8" s="4"/>
+      <c r="DM8" s="4"/>
+      <c r="DN8" s="4"/>
+      <c r="DO8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -2283,25 +2351,25 @@
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
-      <c r="K9" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L9" s="4" t="s">
-        <v>151</v>
-      </c>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
-      <c r="O9" s="4" t="s">
-        <v>152</v>
-      </c>
+      <c r="O9" s="4"/>
       <c r="P9" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="Q9" s="4"/>
+        <v>127</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>156</v>
+      </c>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
-      <c r="T9" s="4"/>
-      <c r="U9" s="4"/>
+      <c r="T9" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="U9" s="4" t="s">
+        <v>158</v>
+      </c>
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
       <c r="X9" s="4"/>
@@ -2395,10 +2463,15 @@
       <c r="DH9" s="4"/>
       <c r="DI9" s="4"/>
       <c r="DJ9" s="4"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK9" s="4"/>
+      <c r="DL9" s="4"/>
+      <c r="DM9" s="4"/>
+      <c r="DN9" s="4"/>
+      <c r="DO9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -2409,25 +2482,25 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
-      <c r="K10" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>154</v>
-      </c>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
-      <c r="O10" s="4" t="s">
-        <v>155</v>
-      </c>
+      <c r="O10" s="4"/>
       <c r="P10" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="Q10" s="4"/>
+        <v>127</v>
+      </c>
+      <c r="Q10" s="4" t="s">
+        <v>159</v>
+      </c>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
-      <c r="T10" s="4"/>
-      <c r="U10" s="4"/>
+      <c r="T10" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="U10" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="V10" s="4"/>
       <c r="W10" s="4"/>
       <c r="X10" s="4"/>
@@ -2521,6 +2594,11 @@
       <c r="DH10" s="4"/>
       <c r="DI10" s="4"/>
       <c r="DJ10" s="4"/>
+      <c r="DK10" s="4"/>
+      <c r="DL10" s="4"/>
+      <c r="DM10" s="4"/>
+      <c r="DN10" s="4"/>
+      <c r="DO10" s="4"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -2560,7 +2638,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2568,82 +2646,82 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2651,37 +2729,37 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2689,27 +2767,27 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2717,27 +2795,27 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2745,7 +2823,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2753,17 +2831,17 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2771,17 +2849,17 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2789,17 +2867,17 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="8" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="8" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2807,17 +2885,17 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="11" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="8" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="8" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2825,17 +2903,17 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="8" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="8" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2843,17 +2921,17 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="8" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="8" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2861,17 +2939,17 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="8" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="8" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2879,12 +2957,12 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="8" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="8" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2892,67 +2970,67 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="9" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="8" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="8" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="8" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="8" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="8" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="8" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="8" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="8" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="8" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="8" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="8" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="8" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Traigo todo el desarrollo de consumibles
</commit_message>
<xml_diff>
--- a/Backend/TablaCargaMasiva.xlsx
+++ b/Backend/TablaCargaMasiva.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="233">
   <si>
     <t xml:space="preserve">codigo_producto</t>
   </si>
@@ -48,6 +48,21 @@
   </si>
   <si>
     <t xml:space="preserve">nombre_imagen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">articulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedronar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">archivo_esp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">archivo_hds</t>
   </si>
   <si>
     <t xml:space="preserve">activo</t>
@@ -995,8 +1010,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:DJ10"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:DO10"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
@@ -1004,12 +1019,15 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="114" min="15" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="119" min="20" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1052,19 +1070,19 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="2" t="s">
@@ -1355,58 +1373,73 @@
       <c r="DJ1" s="2" t="s">
         <v>113</v>
       </c>
+      <c r="DK1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="DL1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="DM1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="DN1" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="DO1" s="2" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>123</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
-      <c r="N2" s="3" t="s">
-        <v>122</v>
-      </c>
+      <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>126</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
+      <c r="S2" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
       <c r="Y2" s="3"/>
@@ -1499,10 +1532,15 @@
       <c r="DH2" s="3"/>
       <c r="DI2" s="3"/>
       <c r="DJ2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK2" s="3"/>
+      <c r="DL2" s="3"/>
+      <c r="DM2" s="3"/>
+      <c r="DN2" s="3"/>
+      <c r="DO2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -1513,28 +1551,28 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
-      <c r="K3" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>127</v>
-      </c>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
-      <c r="O3" s="4" t="s">
-        <v>128</v>
-      </c>
+      <c r="O3" s="4"/>
       <c r="P3" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
+      <c r="T3" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>135</v>
+      </c>
       <c r="W3" s="4"/>
       <c r="X3" s="4"/>
       <c r="Y3" s="4"/>
@@ -1627,10 +1665,15 @@
       <c r="DH3" s="4"/>
       <c r="DI3" s="4"/>
       <c r="DJ3" s="4"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK3" s="4"/>
+      <c r="DL3" s="4"/>
+      <c r="DM3" s="4"/>
+      <c r="DN3" s="4"/>
+      <c r="DO3" s="4"/>
+    </row>
+    <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -1641,28 +1684,28 @@
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
-      <c r="K4" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>131</v>
-      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
-      <c r="O4" s="4" t="s">
-        <v>132</v>
-      </c>
+      <c r="O4" s="4"/>
       <c r="P4" s="4" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
-      <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
-      <c r="V4" s="4"/>
+      <c r="T4" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="U4" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="V4" s="4" t="s">
+        <v>139</v>
+      </c>
       <c r="W4" s="4"/>
       <c r="X4" s="4"/>
       <c r="Y4" s="4"/>
@@ -1755,10 +1798,15 @@
       <c r="DH4" s="4"/>
       <c r="DI4" s="4"/>
       <c r="DJ4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK4" s="4"/>
+      <c r="DL4" s="4"/>
+      <c r="DM4" s="4"/>
+      <c r="DN4" s="4"/>
+      <c r="DO4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -1769,28 +1817,28 @@
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
-      <c r="K5" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>135</v>
-      </c>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
-      <c r="O5" s="4" t="s">
-        <v>136</v>
-      </c>
+      <c r="O5" s="4"/>
       <c r="P5" s="4" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
+      <c r="T5" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="V5" s="4" t="s">
+        <v>143</v>
+      </c>
       <c r="W5" s="4"/>
       <c r="X5" s="4"/>
       <c r="Y5" s="4"/>
@@ -1883,8 +1931,13 @@
       <c r="DH5" s="4"/>
       <c r="DI5" s="4"/>
       <c r="DJ5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK5" s="4"/>
+      <c r="DL5" s="4"/>
+      <c r="DM5" s="4"/>
+      <c r="DN5" s="4"/>
+      <c r="DO5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1999,57 +2052,62 @@
       <c r="DH6" s="3"/>
       <c r="DI6" s="3"/>
       <c r="DJ6" s="3"/>
+      <c r="DK6" s="3"/>
+      <c r="DL6" s="3"/>
+      <c r="DM6" s="3"/>
+      <c r="DN6" s="3"/>
+      <c r="DO6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>123</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
       <c r="L7" s="3"/>
-      <c r="M7" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>122</v>
-      </c>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
       <c r="O7" s="3" t="s">
-        <v>147</v>
+        <v>127</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>148</v>
+        <v>128</v>
       </c>
       <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
+      <c r="R7" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="S7" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="T7" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="U7" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
@@ -2143,10 +2201,15 @@
       <c r="DH7" s="3"/>
       <c r="DI7" s="3"/>
       <c r="DJ7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK7" s="3"/>
+      <c r="DL7" s="3"/>
+      <c r="DM7" s="3"/>
+      <c r="DN7" s="3"/>
+      <c r="DO7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -2157,25 +2220,25 @@
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
-      <c r="K8" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>149</v>
-      </c>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
-      <c r="O8" s="4" t="s">
-        <v>150</v>
-      </c>
+      <c r="O8" s="4"/>
       <c r="P8" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="Q8" s="4"/>
+        <v>127</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>154</v>
+      </c>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
-      <c r="T8" s="4"/>
-      <c r="U8" s="4"/>
+      <c r="T8" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="U8" s="4" t="s">
+        <v>143</v>
+      </c>
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
       <c r="X8" s="4"/>
@@ -2269,10 +2332,15 @@
       <c r="DH8" s="4"/>
       <c r="DI8" s="4"/>
       <c r="DJ8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK8" s="4"/>
+      <c r="DL8" s="4"/>
+      <c r="DM8" s="4"/>
+      <c r="DN8" s="4"/>
+      <c r="DO8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -2283,25 +2351,25 @@
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
-      <c r="K9" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L9" s="4" t="s">
-        <v>151</v>
-      </c>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
-      <c r="O9" s="4" t="s">
-        <v>152</v>
-      </c>
+      <c r="O9" s="4"/>
       <c r="P9" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="Q9" s="4"/>
+        <v>127</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>156</v>
+      </c>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
-      <c r="T9" s="4"/>
-      <c r="U9" s="4"/>
+      <c r="T9" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="U9" s="4" t="s">
+        <v>158</v>
+      </c>
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
       <c r="X9" s="4"/>
@@ -2395,10 +2463,15 @@
       <c r="DH9" s="4"/>
       <c r="DI9" s="4"/>
       <c r="DJ9" s="4"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="DK9" s="4"/>
+      <c r="DL9" s="4"/>
+      <c r="DM9" s="4"/>
+      <c r="DN9" s="4"/>
+      <c r="DO9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -2409,25 +2482,25 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
-      <c r="K10" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>154</v>
-      </c>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
-      <c r="O10" s="4" t="s">
-        <v>155</v>
-      </c>
+      <c r="O10" s="4"/>
       <c r="P10" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="Q10" s="4"/>
+        <v>127</v>
+      </c>
+      <c r="Q10" s="4" t="s">
+        <v>159</v>
+      </c>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
-      <c r="T10" s="4"/>
-      <c r="U10" s="4"/>
+      <c r="T10" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="U10" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="V10" s="4"/>
       <c r="W10" s="4"/>
       <c r="X10" s="4"/>
@@ -2521,6 +2594,11 @@
       <c r="DH10" s="4"/>
       <c r="DI10" s="4"/>
       <c r="DJ10" s="4"/>
+      <c r="DK10" s="4"/>
+      <c r="DL10" s="4"/>
+      <c r="DM10" s="4"/>
+      <c r="DN10" s="4"/>
+      <c r="DO10" s="4"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -2560,7 +2638,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2568,82 +2646,82 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2651,37 +2729,37 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2689,27 +2767,27 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2717,27 +2795,27 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2745,7 +2823,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2753,17 +2831,17 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2771,17 +2849,17 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2789,17 +2867,17 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="8" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="8" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2807,17 +2885,17 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="11" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="8" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="8" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2825,17 +2903,17 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="8" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="8" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2843,17 +2921,17 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="8" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="8" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2861,17 +2939,17 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="8" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="8" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2879,12 +2957,12 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="8" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="8" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2892,67 +2970,67 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="9" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="8" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="8" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="8" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="8" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="8" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="8" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="8" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="8" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="8" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="8" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="8" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="8" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>